<commit_message>
Add Vietnam destinations data from Google Maps backup
</commit_message>
<xml_diff>
--- a/data/chronological_metrics.xlsx
+++ b/data/chronological_metrics.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,37 +429,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>HitRate@10</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Recall@10</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>MRR@10</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>NDCG@10</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Diversity@10</t>
         </is>
@@ -504,7 +516,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -909,7 +921,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19">
@@ -1179,7 +1191,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="29">
@@ -1206,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="30">
@@ -1584,7 +1596,7 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="44">
@@ -2394,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="74">
@@ -2421,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="75">
@@ -2529,7 +2541,7 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="79">
@@ -2934,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="94">
@@ -2961,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="95">
@@ -3609,7 +3621,7 @@
         <v>0</v>
       </c>
       <c r="G118" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="119">
@@ -3744,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="124">
@@ -3879,7 +3891,7 @@
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="129">
@@ -3906,7 +3918,7 @@
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="130">
@@ -4014,7 +4026,7 @@
         <v>0</v>
       </c>
       <c r="G133" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="134">
@@ -4419,7 +4431,7 @@
         <v>0</v>
       </c>
       <c r="G148" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="149">
@@ -4446,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="G149" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="150">
@@ -4959,7 +4971,7 @@
         <v>0</v>
       </c>
       <c r="G168" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="169">
@@ -5634,7 +5646,7 @@
         <v>0</v>
       </c>
       <c r="G193" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="194">
@@ -5661,7 +5673,7 @@
         <v>0</v>
       </c>
       <c r="G194" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="195">
@@ -5769,7 +5781,7 @@
         <v>0</v>
       </c>
       <c r="G198" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="199">
@@ -6444,7 +6456,7 @@
         <v>0</v>
       </c>
       <c r="G223" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="224">
@@ -6579,7 +6591,7 @@
         <v>0</v>
       </c>
       <c r="G228" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="229">
@@ -6714,7 +6726,7 @@
         <v>0</v>
       </c>
       <c r="G233" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="234">
@@ -6741,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="G234" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="235">
@@ -7119,7 +7131,7 @@
         <v>0</v>
       </c>
       <c r="G248" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="249">
@@ -7389,7 +7401,7 @@
         <v>0</v>
       </c>
       <c r="G258" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="259">
@@ -7794,7 +7806,7 @@
         <v>0</v>
       </c>
       <c r="G273" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="274">
@@ -8199,7 +8211,7 @@
         <v>0</v>
       </c>
       <c r="G288" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="289">
@@ -8874,7 +8886,7 @@
         <v>0</v>
       </c>
       <c r="G313" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="314">
@@ -8901,7 +8913,7 @@
         <v>0</v>
       </c>
       <c r="G314" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="315">
@@ -9009,7 +9021,7 @@
         <v>0</v>
       </c>
       <c r="G318" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="319">
@@ -9036,7 +9048,7 @@
         <v>0</v>
       </c>
       <c r="G319" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="320">
@@ -9144,7 +9156,7 @@
         <v>0</v>
       </c>
       <c r="G323" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="324">
@@ -9414,7 +9426,7 @@
         <v>0</v>
       </c>
       <c r="G333" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="334">
@@ -9441,7 +9453,7 @@
         <v>0</v>
       </c>
       <c r="G334" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="335">
@@ -9684,7 +9696,7 @@
         <v>0</v>
       </c>
       <c r="G343" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="344">
@@ -10359,7 +10371,7 @@
         <v>0</v>
       </c>
       <c r="G368" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="369">
@@ -10386,7 +10398,7 @@
         <v>0</v>
       </c>
       <c r="G369" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="370">
@@ -10629,7 +10641,7 @@
         <v>0</v>
       </c>
       <c r="G378" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="379">
@@ -10764,7 +10776,7 @@
         <v>0</v>
       </c>
       <c r="G383" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="384">
@@ -10791,7 +10803,7 @@
         <v>0</v>
       </c>
       <c r="G384" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="385">
@@ -11034,7 +11046,7 @@
         <v>0</v>
       </c>
       <c r="G393" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="394">
@@ -11061,7 +11073,7 @@
         <v>0</v>
       </c>
       <c r="G394" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="395">
@@ -11574,7 +11586,7 @@
         <v>0</v>
       </c>
       <c r="G413" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="414">
@@ -11709,7 +11721,7 @@
         <v>0</v>
       </c>
       <c r="G418" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="419">
@@ -11844,7 +11856,7 @@
         <v>0</v>
       </c>
       <c r="G423" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="424">
@@ -11979,7 +11991,7 @@
         <v>0</v>
       </c>
       <c r="G428" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="429">
@@ -12519,7 +12531,7 @@
         <v>0</v>
       </c>
       <c r="G448" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="449">
@@ -12546,7 +12558,7 @@
         <v>0</v>
       </c>
       <c r="G449" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="450">
@@ -12654,7 +12666,7 @@
         <v>0</v>
       </c>
       <c r="G453" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="454">
@@ -12789,7 +12801,7 @@
         <v>0</v>
       </c>
       <c r="G458" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="459">
@@ -12924,7 +12936,7 @@
         <v>0</v>
       </c>
       <c r="G463" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="464">
@@ -12951,7 +12963,7 @@
         <v>0</v>
       </c>
       <c r="G464" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="465">
@@ -13194,7 +13206,7 @@
         <v>0</v>
       </c>
       <c r="G473" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="474">
@@ -13734,7 +13746,7 @@
         <v>0</v>
       </c>
       <c r="G493" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="494">
@@ -13761,7 +13773,7 @@
         <v>0</v>
       </c>
       <c r="G494" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="495">
@@ -14004,7 +14016,7 @@
         <v>0</v>
       </c>
       <c r="G503" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="504">
@@ -14409,7 +14421,7 @@
         <v>0</v>
       </c>
       <c r="G518" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="519">
@@ -14814,7 +14826,7 @@
         <v>0</v>
       </c>
       <c r="G533" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="534">
@@ -14949,7 +14961,7 @@
         <v>0</v>
       </c>
       <c r="G538" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="539">
@@ -14976,7 +14988,7 @@
         <v>0</v>
       </c>
       <c r="G539" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="540">
@@ -15759,7 +15771,7 @@
         <v>0</v>
       </c>
       <c r="G568" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="569">
@@ -16164,7 +16176,7 @@
         <v>0</v>
       </c>
       <c r="G583" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="584">
@@ -16299,7 +16311,7 @@
         <v>0</v>
       </c>
       <c r="G588" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="589">
@@ -16326,7 +16338,7 @@
         <v>0</v>
       </c>
       <c r="G589" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="590">
@@ -16434,7 +16446,7 @@
         <v>0</v>
       </c>
       <c r="G593" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="594">

</xml_diff>